<commit_message>
Update(Invoke Python): Update the module and call to invoke python to modern invoke
</commit_message>
<xml_diff>
--- a/Archivos/FORMATOS/31.xlsx
+++ b/Archivos/FORMATOS/31.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\FORMATOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA26E77-4975-40E3-A58D-A8D92E929EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51742639-A964-480C-92E4-89CE8EC3DD98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="7" xr2:uid="{4A794D74-3375-41D3-9193-B22F183FDDB6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4A794D74-3375-41D3-9193-B22F183FDDB6}"/>
   </bookViews>
   <sheets>
     <sheet name="01" sheetId="33" r:id="rId1"/>

</xml_diff>